<commit_message>
Dashboard icon navigator is done and added to all pages
</commit_message>
<xml_diff>
--- a/Day 7/Day07.xlsx
+++ b/Day 7/Day07.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C32CE9EF-CDA5-4BF1-97A3-095048362D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1E7C27-FCB8-40DF-AE74-A727E90A4D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{810B916D-8AC5-B94F-AAD8-02E834047D22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{810B916D-8AC5-B94F-AAD8-02E834047D22}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -391,6 +391,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Graphic 2" descr="Table with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85CB3B72-64CC-2DE6-CDBD-70F9B4FD4634}"/>
@@ -402,13 +403,13 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
             <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId3"/>
             </a:ext>
           </a:extLst>
         </a:blip>
@@ -443,6 +444,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Graphic 4" descr="Presentation with pie chart with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D01A2EF3-BC44-E680-3108-A9F85AB3987D}"/>
@@ -454,13 +456,13 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
             <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId4"/>
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId6"/>
             </a:ext>
           </a:extLst>
         </a:blip>
@@ -496,6 +498,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Graphic 6" descr="Envelope with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7ABC13E7-7206-1C4E-E33B-11057ED8DBB2}"/>
@@ -507,13 +510,13 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
             <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId6"/>
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId9"/>
             </a:ext>
           </a:extLst>
         </a:blip>
@@ -533,25 +536,31 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>205740</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:colOff>182879</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>110005</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>581844</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>10344</xdr:rowOff>
+      <xdr:colOff>646854</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>171814</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="Graphic 15" descr="Question Mark with solid fill">
+        <xdr:cNvPr id="2" name="Graphic 1" descr="Table with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9AE1C702-A456-442D-AB92-5ECBF2336390}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC951559-8EE3-453C-9397-3A2F0919D1DA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -560,13 +569,13 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
             <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId8"/>
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId3"/>
             </a:ext>
           </a:extLst>
         </a:blip>
@@ -575,8 +584,282 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="205740" y="3002280"/>
-          <a:ext cx="376104" cy="376104"/>
+          <a:off x="182879" y="1694965"/>
+          <a:ext cx="463975" cy="458049"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>185569</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>75630</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>654801</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>138753</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Graphic 2" descr="Presentation with pie chart with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0AD8F5E8-EF76-4FD8-BC0B-1391257502B4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId6"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="185569" y="1066230"/>
+          <a:ext cx="469232" cy="459363"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>164402</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>163829</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>633634</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>24554</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Graphic 3" descr="Envelope with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3ACD739A-9541-4DEF-A764-E2FEBE87A16B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId9"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="164402" y="2343149"/>
+          <a:ext cx="469232" cy="455085"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>182879</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>110005</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>646854</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>171814</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Graphic 1" descr="Table with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D45FCAC0-9C0D-41B9-9F68-6160B00283F2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId3"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="182879" y="1694965"/>
+          <a:ext cx="463975" cy="458049"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>185569</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>75630</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>654801</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>138753</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Graphic 2" descr="Presentation with pie chart with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB49A192-EAED-488B-BA52-66776E730DD8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId6"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="185569" y="1066230"/>
+          <a:ext cx="469232" cy="459363"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>164402</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>163829</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>633634</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>24554</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Graphic 3" descr="Envelope with solid fill">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{81580875-BF34-460A-BC05-0865F0967D93}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId9"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="164402" y="2343149"/>
+          <a:ext cx="469232" cy="455085"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -886,10 +1169,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32D62819-44D1-EE4C-940E-0D3D0CCB2ED3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.875" style="1"/>
-    <col min="2" max="16384" width="10.875" style="2"/>
+    <col min="1" max="1" width="10.8984375" style="1"/>
+    <col min="2" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -899,18 +1182,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FC16DE6-AF43-5D41-92D8-941949992132}">
-  <dimension ref="C2:K24"/>
-  <sheetFormatPr defaultColWidth="11.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:K24"/>
+  <sheetFormatPr defaultColWidth="11.09765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.875" customWidth="1"/>
+    <col min="1" max="1" width="10.8984375" style="1"/>
     <col min="2" max="2" width="4" customWidth="1"/>
-    <col min="3" max="3" width="14.125" customWidth="1"/>
-    <col min="4" max="4" width="8.625" customWidth="1"/>
-    <col min="5" max="5" width="10.125" customWidth="1"/>
-    <col min="7" max="7" width="12.375" customWidth="1"/>
+    <col min="3" max="3" width="14.09765625" customWidth="1"/>
+    <col min="4" max="4" width="8.59765625" customWidth="1"/>
+    <col min="5" max="5" width="10.09765625" customWidth="1"/>
+    <col min="7" max="7" width="12.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C2" s="11" t="s">
         <v>53</v>
       </c>
@@ -922,7 +1205,7 @@
       <c r="I2" s="11"/>
       <c r="J2" s="11"/>
     </row>
-    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C4" s="5" t="s">
         <v>50</v>
       </c>
@@ -942,7 +1225,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>47</v>
       </c>
@@ -962,7 +1245,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>48</v>
       </c>
@@ -982,7 +1265,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>51</v>
       </c>
@@ -1005,7 +1288,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="8" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>52</v>
       </c>
@@ -1028,7 +1311,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C10" s="11" t="s">
         <v>54</v>
       </c>
@@ -1042,7 +1325,7 @@
       </c>
       <c r="K10" s="11"/>
     </row>
-    <row r="12" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C12" s="4" t="s">
         <v>8</v>
       </c>
@@ -1065,7 +1348,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
         <v>9</v>
       </c>
@@ -1088,7 +1371,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="14" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
         <v>10</v>
       </c>
@@ -1111,7 +1394,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="15" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C15" t="s">
         <v>11</v>
       </c>
@@ -1134,7 +1417,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="16" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C16" t="s">
         <v>12</v>
       </c>
@@ -1157,7 +1440,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="17" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C17" t="s">
         <v>7</v>
       </c>
@@ -1180,7 +1463,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C18" t="s">
         <v>13</v>
       </c>
@@ -1197,7 +1480,7 @@
         <v>253.6</v>
       </c>
     </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
         <v>14</v>
       </c>
@@ -1214,7 +1497,7 @@
         <v>387.5</v>
       </c>
     </row>
-    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
         <v>15</v>
       </c>
@@ -1225,7 +1508,7 @@
         <v>200.6</v>
       </c>
     </row>
-    <row r="21" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
         <v>16</v>
       </c>
@@ -1236,7 +1519,7 @@
         <v>210.6</v>
       </c>
     </row>
-    <row r="22" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C22" t="s">
         <v>17</v>
       </c>
@@ -1247,7 +1530,7 @@
         <v>216.4</v>
       </c>
     </row>
-    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C23" t="s">
         <v>18</v>
       </c>
@@ -1258,7 +1541,7 @@
         <v>222.3</v>
       </c>
     </row>
-    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C24" t="s">
         <v>19</v>
       </c>
@@ -1271,21 +1554,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{604A435B-AFC0-4775-ADA4-3BA01B02C73F}">
-  <dimension ref="C2:E9"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:E9"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.875" customWidth="1"/>
-    <col min="2" max="2" width="4.375" customWidth="1"/>
-    <col min="4" max="4" width="16.625" customWidth="1"/>
+    <col min="1" max="1" width="10.8984375" style="1"/>
+    <col min="2" max="2" width="4.3984375" customWidth="1"/>
+    <col min="4" max="4" width="16.59765625" customWidth="1"/>
     <col min="5" max="5" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
       <c r="C2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1296,7 +1581,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>1</v>
       </c>
@@ -1307,7 +1592,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>4</v>
       </c>
@@ -1318,7 +1603,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>22</v>
       </c>
@@ -1329,7 +1614,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>5</v>
       </c>
@@ -1340,7 +1625,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>6</v>
       </c>
@@ -1351,7 +1636,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>3</v>
       </c>
@@ -1362,7 +1647,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
         <v>2</v>
       </c>
@@ -1384,5 +1669,6 @@
     <hyperlink ref="E9" r:id="rId7" xr:uid="{1E38756C-5E74-4FCB-980C-CE9D026A5A10}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dashboard Layout is made
</commit_message>
<xml_diff>
--- a/Day 7/Day07.xlsx
+++ b/Day 7/Day07.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1E7C27-FCB8-40DF-AE74-A727E90A4D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B61A1E-5BEC-49EE-90CD-F69D8AF59933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{810B916D-8AC5-B94F-AAD8-02E834047D22}"/>
   </bookViews>
@@ -534,6 +534,488 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Rectangle: Rounded Corners 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2F4AD2E6-01A9-859A-D005-C2EFC5791765}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="906780" y="45720"/>
+          <a:ext cx="10271760" cy="670560"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="073673"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:schemeClr val="accent5"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:fillRef>
+        <a:effectRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2800">
+              <a:latin typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:ea typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:cs typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>Sales Analysis Dashboard</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>358140</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>373380</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Rectangle: Rounded Corners 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77A80883-72ED-E92C-DCD4-CE97CD300D63}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7833360" y="853440"/>
+          <a:ext cx="3337560" cy="1226820"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:schemeClr val="accent5"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:fillRef>
+        <a:effectRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400">
+              <a:latin typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:ea typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:cs typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t># of Customer</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>236220</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="Rectangle: Rounded Corners 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9EEEB556-D61B-C6C8-C36D-CCFF70E1239B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4396740" y="845820"/>
+          <a:ext cx="3314700" cy="1226820"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:schemeClr val="accent5"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:fillRef>
+        <a:effectRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400">
+              <a:latin typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:ea typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:cs typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>Profit</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="Rectangle: Rounded Corners 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4D6D3809-D3B2-4EEC-5FC0-D7F2A5049B67}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="914400" y="853440"/>
+          <a:ext cx="3345180" cy="1226820"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:schemeClr val="accent5"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:fillRef>
+        <a:effectRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400">
+              <a:latin typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:ea typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:cs typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>Sales</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>502920</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>769620</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="Rectangle: Rounded Corners 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B10D106-1169-888D-8B45-504980EBFF14}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11300460" y="121920"/>
+          <a:ext cx="2758440" cy="5257800"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="val 3407"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="073673"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:schemeClr val="accent5"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:fillRef>
+        <a:effectRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400">
+              <a:latin typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:ea typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:cs typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>Sales by Region</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>358140</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>373380</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="Rectangle: Rounded Corners 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B485C04D-CD57-9959-3E43-A91BB18C5DDC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7833360" y="2225040"/>
+          <a:ext cx="3337560" cy="2918460"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="val 4918"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:schemeClr val="accent5"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:fillRef>
+        <a:effectRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400">
+              <a:latin typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:ea typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:cs typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>Client Satisfaction</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="Rectangle: Rounded Corners 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD178237-33F5-177D-1B0D-27BE7D333B53}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="914400" y="2225040"/>
+          <a:ext cx="6804660" cy="2918460"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="val 4918"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:schemeClr val="accent5"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:fillRef>
+        <a:effectRef idx="3">
+          <a:schemeClr val="accent5"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400">
+              <a:latin typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:ea typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+              <a:cs typeface="ADLaM Display" panose="020B0604020202020204" pitchFamily="2" charset="0"/>
+            </a:rPr>
+            <a:t>Client Satisfaction</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>

</xml_diff>